<commit_message>
a little adjustment of files
</commit_message>
<xml_diff>
--- a/Src/Assets/StreamingAssets/Common/Tables/Tables/RougeMap.xlsx
+++ b/Src/Assets/StreamingAssets/Common/Tables/Tables/RougeMap.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="32">
   <si>
     <t>Key</t>
   </si>
@@ -45,27 +45,6 @@
   </si>
   <si>
     <t>Possibility</t>
-  </si>
-  <si>
-    <t>Boss</t>
-  </si>
-  <si>
-    <t>Elite</t>
-  </si>
-  <si>
-    <t>精英</t>
-  </si>
-  <si>
-    <t>Sanctuary</t>
-  </si>
-  <si>
-    <t>庇护所</t>
-  </si>
-  <si>
-    <t>Soul Spring</t>
-  </si>
-  <si>
-    <t>灵魂之泉</t>
   </si>
   <si>
     <t>Minion</t>
@@ -1117,7 +1096,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="27.5454545454545" customWidth="1"/>
@@ -1158,93 +1137,93 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>-2</v>
+      </c>
+      <c r="F2">
         <v>1</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>-1</v>
+      </c>
+      <c r="F4">
         <v>1</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
         <v>1</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -1252,19 +1231,19 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="F7">
         <v>0.5</v>
@@ -1272,221 +1251,141 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D9">
         <v>0</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
         <v>1</v>
-      </c>
-      <c r="F11">
-        <v>0.5</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12">
-        <v>0.66</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D13">
         <v>0</v>
       </c>
       <c r="E13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F13">
-        <v>0.66</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D14">
         <v>0</v>
       </c>
       <c r="E14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F14">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="A15" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15">
-        <v>3</v>
-      </c>
-      <c r="F15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" t="s">
-        <v>33</v>
-      </c>
-      <c r="C16" t="s">
-        <v>34</v>
-      </c>
-      <c r="D16">
-        <v>0</v>
-      </c>
-      <c r="E16">
-        <v>3</v>
-      </c>
-      <c r="F16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" t="s">
-        <v>35</v>
-      </c>
-      <c r="B17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17">
-        <v>4</v>
-      </c>
-      <c r="F17">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" t="s">
-        <v>37</v>
-      </c>
-      <c r="B18" t="s">
-        <v>37</v>
-      </c>
-      <c r="C18" t="s">
-        <v>38</v>
-      </c>
-      <c r="D18">
-        <v>0</v>
-      </c>
-      <c r="E18">
-        <v>4</v>
-      </c>
-      <c r="F18">
         <v>0.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
a lot of things 2
</commit_message>
<xml_diff>
--- a/Src/Assets/StreamingAssets/Common/Tables/Tables/RougeMap.xlsx
+++ b/Src/Assets/StreamingAssets/Common/Tables/Tables/RougeMap.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="12080" activeTab="2"/>
+    <workbookView windowWidth="25600" windowHeight="12080" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="RougeMap" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="91">
   <si>
     <t>Key</t>
   </si>
@@ -136,18 +136,6 @@
     <t>Type</t>
   </si>
   <si>
-    <t>1-1</t>
-  </si>
-  <si>
-    <t>["Clumsy Gunner", "Clumsy Gunner", "Clumsy Gunner"]</t>
-  </si>
-  <si>
-    <t>1-2</t>
-  </si>
-  <si>
-    <t>["Mountain Bandit Cluster", "Mountain Bandit Cluster", "Mountain Bandit Cluster", "Mountain Bandit Cluster"]</t>
-  </si>
-  <si>
     <t>1-3</t>
   </si>
   <si>
@@ -232,7 +220,7 @@
     <t>1-16</t>
   </si>
   <si>
-    <t>["Bandit Leader", "Clumsy Gunner", "Clumsy Gunner", "Mountain Bandit Cluster"]</t>
+    <t>["Bandit Leader", "Crow"]</t>
   </si>
   <si>
     <t>1-17</t>
@@ -241,25 +229,13 @@
     <t>["Troll"]</t>
   </si>
   <si>
-    <t>1-18</t>
-  </si>
-  <si>
-    <t>["Bronze Guardian", "Bronze Imp", "Bronze Imp", "Bronze Imp"]</t>
+    <t>1-20</t>
+  </si>
+  <si>
+    <t>["Formless Water", "Formless Water", "Formless Water", "Formless Water"]</t>
   </si>
   <si>
     <t>Boss</t>
-  </si>
-  <si>
-    <t>1-19</t>
-  </si>
-  <si>
-    <t>["Ancient Tree"]</t>
-  </si>
-  <si>
-    <t>1-20</t>
-  </si>
-  <si>
-    <t>["Formless Water", "Formless Water", "Formless Water", "Formless Water"]</t>
   </si>
   <si>
     <t>1-21</t>
@@ -1650,7 +1626,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="4"/>
   <cols>
     <col min="3" max="3" width="116.109090909091" customWidth="1"/>
@@ -1856,44 +1832,44 @@
         <v>56</v>
       </c>
       <c r="D12" s="4">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="E12" t="s">
-        <v>6</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="6">
+        <v>100</v>
+      </c>
+      <c r="E13" t="s">
         <v>57</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="D13" s="6">
-        <v>20</v>
-      </c>
-      <c r="E13" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D14" s="4">
         <v>100</v>
       </c>
       <c r="E14" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1910,7 +1886,7 @@
         <v>100</v>
       </c>
       <c r="E15" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1927,7 +1903,7 @@
         <v>100</v>
       </c>
       <c r="E16" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1941,112 +1917,44 @@
         <v>67</v>
       </c>
       <c r="D17" s="6">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" s="4">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
         <v>68</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D18" s="4">
-        <v>100</v>
-      </c>
-      <c r="E18" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D19" s="6">
         <v>0</v>
       </c>
       <c r="E19" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D20" s="4">
-        <v>0</v>
-      </c>
-      <c r="E20" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="D21" s="6">
-        <v>0</v>
-      </c>
-      <c r="E21" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="D22" s="4">
-        <v>0</v>
-      </c>
-      <c r="E22" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="D23" s="6">
-        <v>0</v>
-      </c>
-      <c r="E23" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -2080,10 +1988,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E1" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -2097,78 +2005,78 @@
         <v>25</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="E2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E3" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>27</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="E4" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C5" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="D5" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="E5" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C6" t="s">
         <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="E6" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>